<commit_message>
Group A hand map round 2 + JIC end transfer: stage now 44 new configurations, checks clean
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PJcT2926CUEincCxCV1ZSx
</commit_message>
<xml_diff>
--- a/tools/_out/brennancad_20261021/regen/stage/straight/DesignTable_5406C_SW2.xlsx
+++ b/tools/_out/brennancad_20261021/regen/stage/straight/DesignTable_5406C_SW2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -906,47 +906,47 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5406-C-4</t>
+          <t>5406-C-24</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.92</v>
+        <v>1.54</v>
       </c>
       <c r="C7" t="n">
-        <v>0.43301</v>
+        <v>1.37121</v>
       </c>
       <c r="D7" t="n">
-        <v>0.75</v>
+        <v>2.375</v>
       </c>
       <c r="E7" t="n">
-        <v>0.43</v>
+        <v>1.72</v>
       </c>
       <c r="F7" t="n">
-        <v>0.67</v>
+        <v>1.16</v>
       </c>
       <c r="G7" t="n">
-        <v>0.43</v>
+        <v>1.72</v>
       </c>
       <c r="H7" t="n">
-        <v>0.67</v>
+        <v>1.16</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0556</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>0.215</v>
+        <v>0.86</v>
       </c>
       <c r="K7" t="n">
-        <v>0.2594</v>
+        <v>0.9296</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>5406-C-4</t>
+          <t>5406-C-24</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Female Pipe Cap (NPTF), 1/4-18 NPTF (female)</t>
+          <t>Female Pipe Cap (NPTF), 1 1/2-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>1/4-18 NPTF (female)</t>
+          <t>1 1/2-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -971,87 +971,251 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Air-Way s87 only (double-pass 6 rows); female NPTF per ANSI B1.20.3 | MODEL: female NPTF port: Air-Way tap drill to MS51503 P1 max per pipe dash (2405 table; Brennan 5405-08-08 STEP VERIFIED -08 only), helical thread over P1; closed hex cap, hex over the full length (ASSUMPTION - cap crown shape unpublished), end chamfers NOT modelled</t>
+          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: THDMAJ_A@DRIVE, L@DRIVE, C1HEX@HEX] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: female NPTF port: Air-Way tap drill to MS51503 P1 max per pipe dash (2405 table; Brennan 5405-08-08 STEP VERIFIED -08 only), helical thread over P1; closed hex cap, hex over the full length (ASSUMPTION - cap crown shape unpublished), end chamfers NOT modelled</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | Brennan CAD record 5406-C-24 (PARTcommunity / CADENAS, THDMAJ_A@DRIVE=A1THD, L@DRIVE=L, C1HEX@HEX=C; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -24 1.72 (A1, A9: Brennan 5405-24-24 / -32-32 STEPs 1.734 / 2.218 -&gt; nearest Air-Way 1.72 / 2.20)</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>5406-C-04</t>
+          <t>5406-C-24</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>5406-C-32</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.65988</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.875</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.1696</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>5406-C-32</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Female Pipe Cap (NPTF), 2-11 1/2 NPTF (female)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>5406C</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2-11 1/2 NPTF (female)</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>plug head</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: THDMAJ_A@DRIVE, L@DRIVE, C1HEX@HEX] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: female NPTF port: Air-Way tap drill to MS51503 P1 max per pipe dash (2405 table; Brennan 5405-08-08 STEP VERIFIED -08 only), helical thread over P1; closed hex cap, hex over the full length (ASSUMPTION - cap crown shape unpublished), end chamfers NOT modelled</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | Brennan CAD record 5406-C-32 (PARTcommunity / CADENAS, THDMAJ_A@DRIVE=A1THD, L@DRIVE=L, C1HEX@HEX=C; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -32 2.2 (A1, A9: Brennan 5405-24-24 / -32-32 STEPs 1.734 / 2.218 -&gt; nearest Air-Way 1.72 / 2.20)</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>5406-C-32</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5406-C-4</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.43301</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.0556</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.2594</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>5406-C-4</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Female Pipe Cap (NPTF), 1/4-18 NPTF (female)</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>5406C</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>1/4-18 NPTF (female)</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>plug head</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Air-Way s87 only (double-pass 6 rows); female NPTF per ANSI B1.20.3 | MODEL: female NPTF port: Air-Way tap drill to MS51503 P1 max per pipe dash (2405 table; Brennan 5405-08-08 STEP VERIFIED -08 only), helical thread over P1; closed hex cap, hex over the full length (ASSUMPTION - cap crown shape unpublished), end chamfers NOT modelled</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>5406-C-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>5406-C-6</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B10" t="n">
         <v>0.97</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C10" t="n">
         <v>0.50807</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D10" t="n">
         <v>0.88</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E10" t="n">
         <v>0.57</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F10" t="n">
         <v>0.68</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G10" t="n">
         <v>0.57</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H10" t="n">
         <v>0.68</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I10" t="n">
         <v>0.0556</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J10" t="n">
         <v>0.285</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K10" t="n">
         <v>0.3294</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>5406-C-6</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Female Pipe Cap (NPTF), 3/8-18 NPTF (female)</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>5406C</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>3/8-18 NPTF (female)</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>plug head</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>Air-Way s87 only (double-pass 6 rows); female NPTF per ANSI B1.20.3 | MODEL: female NPTF port: Air-Way tap drill to MS51503 P1 max per pipe dash (2405 table; Brennan 5405-08-08 STEP VERIFIED -08 only), helical thread over P1; closed hex cap, hex over the full length (ASSUMPTION - cap crown shape unpublished), end chamfers NOT modelled</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>5406-C-06</t>
         </is>

</xml_diff>